<commit_message>
Bench workbook: ladder rungs 2, 4 and 5 marks; README rung status
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bellTesting.xlsx
+++ b/bellTesting.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_claude\KnurLogger\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5122CAB5-9152-461B-9958-C9A42CFF916E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B18D8277-DC67-4B80-9DE8-7C5BBECBB6ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="3210" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{92A98008-AB08-47F0-8EE8-B470B5852900}"/>
+    <workbookView xWindow="38280" yWindow="3210" windowWidth="29040" windowHeight="16440" xr2:uid="{92A98008-AB08-47F0-8EE8-B470B5852900}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="39">
   <si>
     <t>bell:</t>
   </si>
@@ -138,6 +138,12 @@
   </si>
   <si>
     <t>P4L</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>submersion</t>
   </si>
 </sst>
 </file>
@@ -148,7 +154,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -160,6 +166,14 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -221,7 +235,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -238,6 +252,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Calculation" xfId="1" builtinId="22"/>
@@ -553,7 +569,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5764033C-8C05-41CC-A0E2-13CD2D58CEDE}">
-  <dimension ref="A1:AA74"/>
+  <dimension ref="A1:AC75"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -2496,7 +2512,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="65" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="6" t="s">
         <v>0</v>
       </c>
@@ -2560,7 +2576,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="66" spans="1:27" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:29" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B66" t="s">
         <v>13</v>
       </c>
@@ -2592,277 +2608,467 @@
         <v>22</v>
       </c>
     </row>
-    <row r="68" spans="1:27" ht="30" x14ac:dyDescent="0.25">
-      <c r="A68" s="9" t="s">
+    <row r="68" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>37</v>
+      </c>
+      <c r="B68" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B68" t="s">
+      <c r="C68" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D68" t="s">
         <v>27</v>
       </c>
-      <c r="C68" t="s">
+      <c r="E68" t="s">
         <v>28</v>
       </c>
-      <c r="D68" t="s">
+      <c r="F68" t="s">
         <v>29</v>
       </c>
-      <c r="E68" t="s">
+      <c r="G68" t="s">
         <v>30</v>
       </c>
-      <c r="F68" t="s">
+      <c r="H68" t="s">
         <v>31</v>
       </c>
-      <c r="G68" t="s">
+      <c r="I68" t="s">
         <v>32</v>
       </c>
-      <c r="H68" t="s">
+      <c r="J68" t="s">
         <v>33</v>
       </c>
-      <c r="I68" t="s">
+      <c r="K68" t="s">
         <v>34</v>
       </c>
-      <c r="J68" t="s">
+      <c r="L68" t="s">
         <v>35</v>
       </c>
-      <c r="K68" t="s">
+      <c r="M68" t="s">
         <v>36</v>
       </c>
-      <c r="M68" t="s">
+      <c r="O68" t="s">
         <v>27</v>
       </c>
-      <c r="N68" t="s">
+      <c r="P68" t="s">
         <v>28</v>
       </c>
-      <c r="O68" t="s">
+      <c r="Q68" t="s">
         <v>29</v>
       </c>
-      <c r="P68" t="s">
+      <c r="R68" t="s">
         <v>30</v>
       </c>
-      <c r="Q68" t="s">
+      <c r="S68" t="s">
         <v>31</v>
       </c>
-      <c r="R68" t="s">
+      <c r="T68" t="s">
         <v>32</v>
       </c>
-      <c r="S68" t="s">
+      <c r="U68" t="s">
         <v>33</v>
       </c>
-      <c r="T68" t="s">
+      <c r="V68" t="s">
         <v>34</v>
       </c>
-      <c r="U68" t="s">
+      <c r="W68" t="s">
         <v>35</v>
       </c>
-      <c r="V68" t="s">
+      <c r="X68" t="s">
         <v>36</v>
       </c>
-      <c r="X68" t="s">
+      <c r="Z68" t="s">
         <v>33</v>
       </c>
-      <c r="Y68" t="s">
+      <c r="AA68" t="s">
         <v>34</v>
       </c>
-      <c r="Z68" t="s">
+      <c r="AB68" t="s">
         <v>35</v>
       </c>
-      <c r="AA68" t="s">
+      <c r="AC68" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="69" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A69">
+    <row r="69" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A69" s="12">
+        <v>46287</v>
+      </c>
+      <c r="B69" s="13">
         <v>98.8</v>
       </c>
-      <c r="B69" s="5">
+      <c r="C69" s="13">
+        <v>70</v>
+      </c>
+      <c r="D69" s="5">
         <v>0.70729166666666665</v>
       </c>
-      <c r="C69" s="5">
+      <c r="E69" s="5">
         <v>0.70821759259259254</v>
       </c>
-      <c r="D69" s="5">
+      <c r="F69" s="5">
         <v>0.70960648148148153</v>
       </c>
-      <c r="E69" s="5">
+      <c r="G69" s="5">
         <v>0.71076388888888886</v>
       </c>
-      <c r="F69" s="5">
+      <c r="H69" s="5">
         <v>0.71174768518518516</v>
       </c>
-      <c r="G69" s="5">
+      <c r="I69" s="5">
         <v>0.71250000000000002</v>
       </c>
-      <c r="H69" s="5">
+      <c r="J69" s="5">
         <v>0.71331018518518519</v>
       </c>
-      <c r="I69" s="5">
+      <c r="K69" s="5">
         <v>0.71400462962962963</v>
       </c>
-      <c r="J69" s="5">
+      <c r="L69" s="5">
         <v>0.71469907407407407</v>
       </c>
-      <c r="K69" s="5">
+      <c r="M69" s="5">
         <v>0.71539351851851851</v>
       </c>
-      <c r="M69" s="5">
+      <c r="O69" s="5">
         <v>0.7309606481481481</v>
       </c>
-      <c r="N69" s="5">
+      <c r="P69" s="5">
         <v>0.73171296296296295</v>
       </c>
-      <c r="O69" s="5">
+      <c r="Q69" s="5">
         <v>0.73298611111111112</v>
       </c>
-      <c r="P69" s="5">
+      <c r="R69" s="5">
         <v>0.73356481481481484</v>
       </c>
-      <c r="Q69" s="5">
+      <c r="S69" s="5">
         <v>0.734375</v>
       </c>
-      <c r="R69" s="5">
+      <c r="T69" s="5">
         <v>0.7354398148148148</v>
       </c>
-      <c r="S69" s="5">
+      <c r="U69" s="5">
         <v>0.73611111111111116</v>
       </c>
-      <c r="T69" s="5">
+      <c r="V69" s="5">
         <v>0.7368055555555556</v>
       </c>
-      <c r="U69" s="5">
+      <c r="W69" s="5">
         <v>0.73784722222222221</v>
       </c>
-      <c r="V69" s="5">
+      <c r="X69" s="5">
         <v>0.73854166666666665</v>
       </c>
-      <c r="X69" s="5">
+      <c r="Z69" s="5">
         <v>0.75567129629629626</v>
       </c>
-      <c r="Y69" s="5">
+      <c r="AA69" s="5">
         <v>0.75694444444444442</v>
       </c>
-      <c r="Z69" s="5">
+      <c r="AB69" s="5">
         <v>0.75798611111111114</v>
       </c>
-      <c r="AA69" s="5">
+      <c r="AC69" s="5">
         <v>0.75868055555555558</v>
       </c>
     </row>
-    <row r="70" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A70">
+    <row r="70" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A70" s="12">
+        <v>46288</v>
+      </c>
+      <c r="B70" s="13">
         <v>174</v>
       </c>
-    </row>
-    <row r="71" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A71">
+      <c r="C70" s="13">
+        <v>70</v>
+      </c>
+      <c r="D70" s="5">
+        <v>0.72027777777777779</v>
+      </c>
+      <c r="E70" s="5">
+        <v>0.72122685185185187</v>
+      </c>
+      <c r="F70" s="5">
+        <v>0.72283564814814816</v>
+      </c>
+      <c r="G70" s="5">
+        <v>0.72501157407407413</v>
+      </c>
+      <c r="H70" s="5">
+        <v>0.72615740740740742</v>
+      </c>
+      <c r="I70" s="5">
+        <v>0.72694444444444439</v>
+      </c>
+      <c r="J70" s="5">
+        <v>0.7283101851851852</v>
+      </c>
+      <c r="K70" s="5">
+        <v>0.72905092592592591</v>
+      </c>
+      <c r="L70" s="5">
+        <v>0.73038194444444449</v>
+      </c>
+      <c r="M70" s="5">
+        <v>0.73199074074074078</v>
+      </c>
+      <c r="O70" s="5">
+        <v>0.75027777777777782</v>
+      </c>
+      <c r="P70" s="5">
+        <v>0.75210648148148151</v>
+      </c>
+      <c r="Q70" s="5">
+        <v>0.75364583333333335</v>
+      </c>
+      <c r="R70" s="5">
+        <v>0.75526620370370368</v>
+      </c>
+    </row>
+    <row r="71" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A71" s="12">
+        <v>46287</v>
+      </c>
+      <c r="B71" s="13">
         <v>244.7</v>
       </c>
-      <c r="B71" s="5">
+      <c r="C71" s="13">
+        <v>70</v>
+      </c>
+      <c r="D71" s="5">
         <v>0.83424768518518522</v>
       </c>
-      <c r="C71" s="5">
+      <c r="E71" s="5">
         <v>0.83879629629629626</v>
       </c>
-      <c r="D71" s="5">
+      <c r="F71" s="5">
         <v>0.84012731481481484</v>
       </c>
-      <c r="E71" s="5">
+      <c r="G71" s="5">
         <v>0.84119212962962964</v>
       </c>
-      <c r="F71" s="5">
+      <c r="H71" s="5">
         <v>0.84537037037037033</v>
       </c>
-      <c r="G71" s="5">
+      <c r="I71" s="5">
         <v>0.8473032407407407</v>
       </c>
-      <c r="H71" s="5">
+      <c r="J71" s="5">
         <v>0.84900462962962964</v>
       </c>
-      <c r="I71" s="5">
+      <c r="K71" s="5">
         <v>0.84996527777777775</v>
       </c>
-      <c r="J71" s="5">
+      <c r="L71" s="5">
         <v>0.85160879629629627</v>
       </c>
-      <c r="K71" s="5">
+      <c r="M71" s="5">
         <v>0.85218749999999999</v>
       </c>
     </row>
-    <row r="72" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A72">
+    <row r="72" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A72" s="12">
+        <v>46288</v>
+      </c>
+      <c r="B72" s="13">
         <v>346.7</v>
       </c>
-      <c r="F72" s="10"/>
-      <c r="G72" s="10"/>
-      <c r="Q72" s="10"/>
-      <c r="R72" s="10"/>
-    </row>
-    <row r="73" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A73">
+      <c r="C72" s="13">
+        <v>70</v>
+      </c>
+      <c r="D72" s="5">
+        <v>0.79984953703703698</v>
+      </c>
+      <c r="E72" s="5">
+        <v>0.80206018518518518</v>
+      </c>
+      <c r="F72" s="5">
+        <v>0.80344907407407407</v>
+      </c>
+      <c r="G72" s="5">
+        <v>0.80447916666666663</v>
+      </c>
+      <c r="H72" s="10"/>
+      <c r="I72" s="10"/>
+      <c r="J72" s="5">
+        <v>0.80541666666666667</v>
+      </c>
+      <c r="K72" s="5">
+        <v>0.80628472222222225</v>
+      </c>
+      <c r="L72" s="5">
+        <v>0.80769675925925921</v>
+      </c>
+      <c r="M72" s="5">
+        <v>0.80914351851851851</v>
+      </c>
+      <c r="Q72" s="5">
+        <v>0.81390046296296292</v>
+      </c>
+      <c r="R72" s="5">
+        <v>0.81460648148148151</v>
+      </c>
+      <c r="S72" s="10"/>
+      <c r="T72" s="10"/>
+      <c r="U72" s="5">
+        <v>0.81574074074074077</v>
+      </c>
+      <c r="V72" s="5">
+        <v>0.81809027777777776</v>
+      </c>
+    </row>
+    <row r="73" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A73" s="12">
+        <v>46288</v>
+      </c>
+      <c r="B73" s="13">
         <v>471.09999999999997</v>
       </c>
-      <c r="F73" s="10"/>
-      <c r="G73" s="10"/>
-      <c r="Q73" s="10"/>
-      <c r="R73" s="10"/>
-    </row>
-    <row r="74" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A74">
+      <c r="C73" s="13">
+        <v>65</v>
+      </c>
+      <c r="D73" s="5">
+        <v>0.84606481481481477</v>
+      </c>
+      <c r="E73" s="5">
+        <v>0.84866898148148151</v>
+      </c>
+      <c r="F73" s="5">
+        <v>0.851099537037037</v>
+      </c>
+      <c r="G73" s="5">
+        <v>0.85575231481481484</v>
+      </c>
+      <c r="H73" s="10"/>
+      <c r="I73" s="10"/>
+      <c r="J73" s="5">
+        <v>0.85804398148148153</v>
+      </c>
+      <c r="K73" s="5">
+        <v>0.86047453703703702</v>
+      </c>
+      <c r="L73" s="5">
+        <v>0.86303240740740739</v>
+      </c>
+      <c r="M73" s="5">
+        <v>0.86525462962962962</v>
+      </c>
+      <c r="R73" s="5">
+        <v>0.87465277777777772</v>
+      </c>
+      <c r="S73" s="10"/>
+      <c r="T73" s="10"/>
+    </row>
+    <row r="74" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A74" s="12">
+        <v>46288</v>
+      </c>
+      <c r="B74" s="13">
+        <v>471.09999999999997</v>
+      </c>
+      <c r="C74" s="13">
+        <v>70</v>
+      </c>
+      <c r="D74" s="5">
+        <v>0.84704861111111107</v>
+      </c>
+      <c r="E74" s="5">
+        <v>0.84953703703703709</v>
+      </c>
+      <c r="F74" s="5">
+        <v>0.85193287037037035</v>
+      </c>
+      <c r="G74" s="5">
+        <v>0.85671296296296295</v>
+      </c>
+      <c r="H74" s="10"/>
+      <c r="I74" s="10"/>
+      <c r="J74" s="5">
+        <v>0.85901620370370368</v>
+      </c>
+      <c r="K74" s="5">
+        <v>0.8613425925925926</v>
+      </c>
+      <c r="L74" s="5">
+        <v>0.86396990740740742</v>
+      </c>
+      <c r="M74" s="5">
+        <v>0.86618055555555551</v>
+      </c>
+      <c r="R74" s="5">
+        <v>0.87561342592592595</v>
+      </c>
+      <c r="S74" s="10"/>
+      <c r="T74" s="10"/>
+    </row>
+    <row r="75" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A75" s="12">
+        <v>46287</v>
+      </c>
+      <c r="B75" s="13">
         <v>728.5</v>
       </c>
-      <c r="B74" s="5">
+      <c r="C75" s="13">
+        <v>70</v>
+      </c>
+      <c r="D75" s="5">
         <v>0.78306712962962965</v>
       </c>
-      <c r="C74" s="5">
+      <c r="E75" s="5">
         <v>0.78408564814814818</v>
       </c>
-      <c r="D74" s="5">
+      <c r="F75" s="5">
         <v>0.78546296296296292</v>
       </c>
-      <c r="E74" s="5">
+      <c r="G75" s="5">
         <v>0.78641203703703699</v>
       </c>
-      <c r="F74" s="10"/>
-      <c r="G74" s="10"/>
-      <c r="H74" s="5">
+      <c r="H75" s="10"/>
+      <c r="I75" s="10"/>
+      <c r="J75" s="5">
         <v>0.78739583333333329</v>
       </c>
-      <c r="I74" s="5">
+      <c r="K75" s="5">
         <v>0.7885416666666667</v>
       </c>
-      <c r="J74" s="5">
+      <c r="L75" s="5">
         <v>0.79045138888888888</v>
       </c>
-      <c r="K74" s="5">
+      <c r="M75" s="5">
         <v>0.79184027777777777</v>
       </c>
-      <c r="M74" s="5">
+      <c r="O75" s="5">
         <v>0.79314814814814816</v>
       </c>
-      <c r="N74" s="5">
+      <c r="P75" s="5">
         <v>0.79402777777777778</v>
       </c>
-      <c r="O74" s="5">
+      <c r="Q75" s="5">
         <v>0.79469907407407403</v>
       </c>
-      <c r="P74" s="5">
+      <c r="R75" s="5">
         <v>0.79539351851851847</v>
       </c>
-      <c r="Q74" s="10"/>
-      <c r="R74" s="10"/>
-      <c r="S74" s="5">
+      <c r="S75" s="10"/>
+      <c r="T75" s="10"/>
+      <c r="U75" s="5">
         <v>0.79625000000000001</v>
       </c>
-      <c r="T74" s="5">
+      <c r="V75" s="5">
         <v>0.79688657407407404</v>
       </c>
-      <c r="U74" s="5">
+      <c r="W75" s="5">
         <v>0.79782407407407407</v>
       </c>
-      <c r="V74" s="5">
+      <c r="X75" s="5">
         <v>0.7988425925925926</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2895,7 +3101,7 @@
         <v>5.7</v>
       </c>
       <c r="D3">
-        <f>B3-C3</f>
+        <f t="shared" ref="D3:D8" si="0">B3-C3</f>
         <v>98.8</v>
       </c>
     </row>
@@ -2907,7 +3113,7 @@
         <v>16.5</v>
       </c>
       <c r="D4">
-        <f>B4-C4</f>
+        <f t="shared" si="0"/>
         <v>174</v>
       </c>
     </row>
@@ -2919,7 +3125,7 @@
         <v>51.5</v>
       </c>
       <c r="D5">
-        <f>B5-C5</f>
+        <f t="shared" si="0"/>
         <v>244.7</v>
       </c>
       <c r="G5" s="2"/>
@@ -2934,7 +3140,7 @@
         <v>39.5</v>
       </c>
       <c r="D6">
-        <f>B6-C6</f>
+        <f t="shared" si="0"/>
         <v>346.7</v>
       </c>
     </row>
@@ -2946,7 +3152,7 @@
         <v>59.2</v>
       </c>
       <c r="D7">
-        <f>B7-C7</f>
+        <f t="shared" si="0"/>
         <v>471.09999999999997</v>
       </c>
     </row>
@@ -2958,7 +3164,7 @@
         <v>95.4</v>
       </c>
       <c r="D8">
-        <f>B8-C8</f>
+        <f t="shared" si="0"/>
         <v>728.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Pressure correction: line-resistance input done; bell workbook update
The correction handoff now points at the measured line-resistance
parameters in ndLouvers pressure-testing.md §3.3a. calibrationBell.md
notes plan open item 57 as closed. bellTesting.xlsx carries the
2026-09-24 line-resistance marks.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bellTesting.xlsx
+++ b/bellTesting.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_claude\KnurLogger\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B18D8277-DC67-4B80-9DE8-7C5BBECBB6ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5391D648-11CE-4480-BEA1-91601F6AF0CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="3210" windowWidth="29040" windowHeight="16440" xr2:uid="{92A98008-AB08-47F0-8EE8-B470B5852900}"/>
+    <workbookView xWindow="38280" yWindow="3210" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{92A98008-AB08-47F0-8EE8-B470B5852900}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="ballasts" sheetId="2" r:id="rId2"/>
+    <sheet name="lineR testing" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="48">
   <si>
     <t>bell:</t>
   </si>
@@ -144,6 +145,33 @@
   </si>
   <si>
     <t>submersion</t>
+  </si>
+  <si>
+    <t>section no</t>
+  </si>
+  <si>
+    <t>mm</t>
+  </si>
+  <si>
+    <t>coupler</t>
+  </si>
+  <si>
+    <t>2.4x27mm</t>
+  </si>
+  <si>
+    <t>rung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rung6(823.9g dry) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rung3(296.2g dry) </t>
+  </si>
+  <si>
+    <t>P0H_noFilterNoWand</t>
+  </si>
+  <si>
+    <t>P0H_LwLine</t>
   </si>
 </sst>
 </file>
@@ -256,8 +284,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Calculation" xfId="1" builtinId="22"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normalny" xfId="0" builtinId="0"/>
+    <cellStyle name="Obliczenia" xfId="1" builtinId="22"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -273,9 +301,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Motyw pakietu Office">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Pakiet Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -313,7 +341,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Pakiet Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -419,7 +447,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Pakiet Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3074,7 +3102,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F08FB72C-BF48-45E5-AFBC-78389EEFAAFD}">
-  <dimension ref="B2:I11"/>
+  <dimension ref="A2:I11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="15.140625" bestFit="1" customWidth="1"/>
@@ -3082,7 +3110,10 @@
     <col min="4" max="4" width="20.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>43</v>
+      </c>
       <c r="B2" t="s">
         <v>23</v>
       </c>
@@ -3093,7 +3124,10 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="13">
+        <v>1</v>
+      </c>
       <c r="B3">
         <v>104.5</v>
       </c>
@@ -3105,7 +3139,10 @@
         <v>98.8</v>
       </c>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="13">
+        <v>2</v>
+      </c>
       <c r="B4">
         <v>190.5</v>
       </c>
@@ -3117,7 +3154,10 @@
         <v>174</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="13">
+        <v>3</v>
+      </c>
       <c r="B5">
         <v>296.2</v>
       </c>
@@ -3132,7 +3172,10 @@
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
     </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="13">
+        <v>4</v>
+      </c>
       <c r="B6">
         <v>386.2</v>
       </c>
@@ -3144,7 +3187,10 @@
         <v>346.7</v>
       </c>
     </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="13">
+        <v>5</v>
+      </c>
       <c r="B7">
         <v>530.29999999999995</v>
       </c>
@@ -3156,7 +3202,10 @@
         <v>471.09999999999997</v>
       </c>
     </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="13">
+        <v>6</v>
+      </c>
       <c r="B8">
         <v>823.9</v>
       </c>
@@ -3168,11 +3217,233 @@
         <v>728.5</v>
       </c>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C11" s="2"/>
       <c r="E11" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{839ABADE-E527-4AD4-983B-2FD78592B3F2}">
+  <dimension ref="A2:L17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="20.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1538</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>8550</v>
+      </c>
+      <c r="D4">
+        <f>C4+C3</f>
+        <v>10088</v>
+      </c>
+      <c r="E4">
+        <f>D4/1000</f>
+        <v>10.087999999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" t="s">
+        <v>31</v>
+      </c>
+      <c r="E9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" s="12">
+        <v>46289</v>
+      </c>
+      <c r="B10">
+        <v>65</v>
+      </c>
+      <c r="C10" s="5">
+        <v>0.59247685185185184</v>
+      </c>
+      <c r="D10" s="5">
+        <v>0.59829861111111116</v>
+      </c>
+      <c r="E10" s="5">
+        <v>0.61707175925925928</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B11">
+        <v>70</v>
+      </c>
+      <c r="C11" s="5">
+        <v>0.59398148148148144</v>
+      </c>
+      <c r="D11" s="5">
+        <v>0.59982638888888884</v>
+      </c>
+      <c r="E11" s="5">
+        <v>0.6186342592592593</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>44</v>
+      </c>
+      <c r="B13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" t="s">
+        <v>47</v>
+      </c>
+      <c r="E13" t="s">
+        <v>46</v>
+      </c>
+      <c r="F13" t="s">
+        <v>29</v>
+      </c>
+      <c r="G13" t="s">
+        <v>33</v>
+      </c>
+      <c r="H13" t="s">
+        <v>35</v>
+      </c>
+      <c r="J13" t="s">
+        <v>29</v>
+      </c>
+      <c r="K13" t="s">
+        <v>33</v>
+      </c>
+      <c r="L13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" s="12">
+        <v>46289</v>
+      </c>
+      <c r="B14">
+        <v>65</v>
+      </c>
+      <c r="C14" s="5">
+        <v>0.6355439814814815</v>
+      </c>
+      <c r="D14" s="5">
+        <v>0.64118055555555553</v>
+      </c>
+      <c r="E14" s="5">
+        <v>0.6441203703703704</v>
+      </c>
+      <c r="F14" s="5">
+        <v>0.65976851851851848</v>
+      </c>
+      <c r="G14" s="5">
+        <v>0.66214120370370366</v>
+      </c>
+      <c r="H14" s="5">
+        <v>0.66421296296296295</v>
+      </c>
+      <c r="J14" s="5">
+        <v>0.68994212962962964</v>
+      </c>
+      <c r="K14" s="5">
+        <v>0.69207175925925923</v>
+      </c>
+      <c r="L14" s="5">
+        <v>0.73559027777777775</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B15">
+        <v>70</v>
+      </c>
+      <c r="C15" s="5">
+        <v>0.6363657407407407</v>
+      </c>
+      <c r="D15" s="5">
+        <v>0.64197916666666666</v>
+      </c>
+      <c r="E15" s="5">
+        <v>0.64490740740740737</v>
+      </c>
+      <c r="F15" s="5">
+        <v>0.6605092592592593</v>
+      </c>
+      <c r="G15" s="5">
+        <v>0.66295138888888894</v>
+      </c>
+      <c r="H15" s="5">
+        <v>0.66497685185185185</v>
+      </c>
+      <c r="J15" s="5">
+        <v>0.69072916666666662</v>
+      </c>
+      <c r="K15" s="5">
+        <v>0.69291666666666663</v>
+      </c>
+      <c r="L15" s="5">
+        <v>0.73631944444444442</v>
+      </c>
+    </row>
+    <row r="17" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="C17" s="5">
+        <f>C15-C14</f>
+        <v>8.2175925925920268E-4</v>
+      </c>
+      <c r="L17" s="5">
+        <f>L15-L14</f>
+        <v>7.2916666666666963E-4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>